<commit_message>
Allow applied corrections and structured budget extraction
</commit_message>
<xml_diff>
--- a/web/public/household-cfo-budget-template.xlsx
+++ b/web/public/household-cfo-budget-template.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Household CFO Budget" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Household CFO Budget'!$A$1:$F$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Household CFO Budget'!$A$1:$G$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -459,7 +459,8 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -490,6 +491,11 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>payment</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>notes</t>
         </is>
       </c>
@@ -518,7 +524,8 @@
           <t>job</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="3" t="n"/>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Demo take-home monthly income</t>
         </is>
@@ -548,7 +555,8 @@
           <t>business</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="3" t="n"/>
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Demo side income</t>
         </is>
@@ -578,7 +586,8 @@
           <t>non_discretionary</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" s="3" t="n"/>
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Fixed housing cost</t>
         </is>
@@ -608,7 +617,8 @@
           <t>non_discretionary</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" s="3" t="n"/>
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Power water internet phone</t>
         </is>
@@ -638,7 +648,8 @@
           <t>discretionary</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F6" s="3" t="n"/>
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Food and household supplies</t>
         </is>
@@ -668,7 +679,8 @@
           <t>discretionary</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F7" s="3" t="n"/>
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Flexible spending to watch</t>
         </is>
@@ -698,7 +710,8 @@
           <t>sinking_expected</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F8" s="3" t="n"/>
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Expected sinking fund</t>
         </is>
@@ -728,7 +741,8 @@
           <t>sinking_unexpected</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F9" s="3" t="n"/>
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Unexpected sinking fund</t>
         </is>
@@ -758,7 +772,8 @@
           <t>emergency_fund</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F10" s="5" t="n"/>
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>Cash reserve balance</t>
         </is>
@@ -788,14 +803,17 @@
           <t>credit_card</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>Minimum payment 175</t>
+      <c r="F11" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>Minimum payment</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F11"/>
+  <autoFilter ref="A1:G11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>